<commit_message>
Alcune correzioni alle condizioni per il calcolo dei ritardi
</commit_message>
<xml_diff>
--- a/PS-VRP/Dati_output/schedulazione_veicoli.xlsx
+++ b/PS-VRP/Dati_output/schedulazione_veicoli.xlsx
@@ -29,7 +29,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -50,12 +50,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
-        <bgColor rgb="00F4CCCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FCE5CD"/>
         <bgColor rgb="00FCE5CD"/>
       </patternFill>
@@ -68,26 +62,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EAD1DC"/>
-        <bgColor rgb="00EAD1DC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00EEEEEE"/>
         <bgColor rgb="00EEEEEE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D2E9"/>
-        <bgColor rgb="00D9D2E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D5E8D4"/>
-        <bgColor rgb="00D5E8D4"/>
+        <fgColor rgb="00F4CCCC"/>
+        <bgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -109,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -133,15 +115,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -509,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B76"/>
+  <dimension ref="A1:B125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -530,205 +503,219 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>252723</v>
+        <v>255699</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>240050</v>
+        <v>40987</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>252207</v>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>240050</v>
+        <v>255672</v>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>40968</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>252680</v>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>240050</v>
+        <v>255072</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>40999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>252210</v>
+        <v>255047</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>240050</v>
+        <v>40987</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>252209</v>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>240050</v>
+        <v>255534</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>40988</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>252371</v>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>240050</v>
+        <v>255244</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>40988</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>243569</v>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>240055</v>
+        <v>255334</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>252814</v>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>309</v>
+        <v>255775</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>252362</v>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>240055</v>
+        <v>254061</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>252378</v>
-      </c>
-      <c r="B11" s="4" t="n">
-        <v>240055</v>
+        <v>260254</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>252298</v>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>302</v>
+        <v>255470</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>40987</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>250383</v>
-      </c>
-      <c r="B13" s="4" t="n">
-        <v>240055</v>
+        <v>254779</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>252495</v>
-      </c>
-      <c r="B14" s="7" t="n">
-        <v>240054</v>
+        <v>255292</v>
+      </c>
+      <c r="B14" s="8" t="n">
+        <v>40991</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>252519</v>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>240055</v>
+        <v>254067</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>252890</v>
-      </c>
-      <c r="B16" s="7" t="n">
-        <v>240054</v>
+        <v>254685</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>251812</v>
-      </c>
-      <c r="B17" s="6" t="n">
-        <v>302</v>
+        <v>255593</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>252369</v>
-      </c>
-      <c r="B18" s="4" t="n">
-        <v>240055</v>
+        <v>255596</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>250284</v>
-      </c>
-      <c r="B19" s="8" t="n">
-        <v>240046</v>
+        <v>255560</v>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>40988</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>252783</v>
-      </c>
-      <c r="B20" s="7" t="n">
-        <v>303</v>
+        <v>255667</v>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>40991</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>252467</v>
-      </c>
-      <c r="B21" s="8" t="n">
-        <v>240046</v>
+        <v>255700</v>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>40987</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>252476</v>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>255354</v>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>40989</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>252665</v>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>255676</v>
+      </c>
+      <c r="B23" s="8" t="n">
+        <v>40991</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>252277</v>
-      </c>
-      <c r="B24" s="7" t="n">
-        <v>40024</v>
+        <v>255765</v>
+      </c>
+      <c r="B24" s="8" t="n">
+        <v>40991</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>252350</v>
-      </c>
-      <c r="B25" s="7" t="n">
-        <v>40055</v>
+        <v>255462</v>
+      </c>
+      <c r="B25" s="8" t="n">
+        <v>40991</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>252598</v>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
+        <v>255802</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -736,9 +723,9 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>252576</v>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
+        <v>251077</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -746,9 +733,9 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>252779</v>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
+        <v>251288</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -756,9 +743,9 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>252899</v>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
+        <v>255397</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -766,9 +753,9 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>252426</v>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
+        <v>255361</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -776,9 +763,9 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>252778</v>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
+        <v>255275</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -786,9 +773,9 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>252157</v>
-      </c>
-      <c r="B32" s="9" t="inlineStr">
+        <v>254914</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -796,123 +783,143 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>252201</v>
-      </c>
-      <c r="B33" s="7" t="n">
-        <v>40055</v>
+        <v>255640</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>252999</v>
-      </c>
-      <c r="B34" s="7" t="n">
-        <v>303</v>
+        <v>254666</v>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>252087</v>
-      </c>
-      <c r="B35" s="5" t="n">
-        <v>307</v>
+        <v>254788</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>251849</v>
-      </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>40042 (esterno)</t>
+        <v>255767</v>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>252220</v>
-      </c>
-      <c r="B37" s="3" t="n">
-        <v>240050</v>
+        <v>255762</v>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>235572</v>
-      </c>
-      <c r="B38" s="4" t="n">
-        <v>240055</v>
+        <v>255764</v>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>244023</v>
-      </c>
-      <c r="B39" s="7" t="n">
-        <v>240054</v>
+        <v>254363</v>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>252638</v>
-      </c>
-      <c r="B40" s="7" t="n">
-        <v>303</v>
+        <v>235572</v>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>252085</v>
-      </c>
-      <c r="B41" s="5" t="n">
-        <v>307</v>
+        <v>255353</v>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>252549</v>
-      </c>
-      <c r="B42" s="3" t="n">
-        <v>240050</v>
+        <v>244023</v>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>252662</v>
-      </c>
-      <c r="B43" s="8" t="n">
-        <v>240046</v>
+        <v>254460</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>252656</v>
-      </c>
-      <c r="B44" s="8" t="n">
-        <v>240046</v>
+        <v>255507</v>
+      </c>
+      <c r="B44" s="6" t="n">
+        <v>40988</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>252473</v>
-      </c>
-      <c r="B45" s="8" t="n">
-        <v>240046</v>
+        <v>255256</v>
+      </c>
+      <c r="B45" s="6" t="n">
+        <v>40988</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>252790</v>
-      </c>
-      <c r="B46" s="10" t="n">
-        <v>240049</v>
+        <v>255780</v>
+      </c>
+      <c r="B46" s="4" t="n">
+        <v>40968</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>252336</v>
-      </c>
-      <c r="B47" s="9" t="inlineStr">
+        <v>255590</v>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -920,179 +927,195 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>252364</v>
-      </c>
-      <c r="B48" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>255568</v>
+      </c>
+      <c r="B48" s="6" t="n">
+        <v>40988</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>252470</v>
-      </c>
-      <c r="B49" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>255698</v>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>40987</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>252334</v>
-      </c>
-      <c r="B50" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>254622</v>
+      </c>
+      <c r="B50" s="8" t="n">
+        <v>40991</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>252713</v>
-      </c>
-      <c r="B51" s="6" t="n">
-        <v>302</v>
+        <v>255441</v>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>252456</v>
-      </c>
-      <c r="B52" s="11" t="n">
-        <v>40049</v>
+        <v>255457</v>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>252755</v>
-      </c>
-      <c r="B53" s="6" t="n">
-        <v>302</v>
+        <v>254112</v>
+      </c>
+      <c r="B53" s="8" t="n">
+        <v>40991</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>251495</v>
-      </c>
-      <c r="B54" s="10" t="n">
-        <v>240049</v>
+        <v>254878</v>
+      </c>
+      <c r="B54" s="8" t="n">
+        <v>40991</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>251926</v>
-      </c>
-      <c r="B55" s="10" t="n">
-        <v>240049</v>
+        <v>254997</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>252414</v>
-      </c>
-      <c r="B56" s="7" t="n">
-        <v>240054</v>
+        <v>253133</v>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>252511</v>
-      </c>
-      <c r="B57" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>255707</v>
+      </c>
+      <c r="B57" s="8" t="n">
+        <v>40991</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>252507</v>
-      </c>
-      <c r="B58" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>255696</v>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>40987</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>252978</v>
-      </c>
-      <c r="B59" s="11" t="n">
-        <v>40049</v>
+        <v>255391</v>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>251919</v>
-      </c>
-      <c r="B60" s="6" t="n">
-        <v>302</v>
+        <v>252647</v>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>252245</v>
-      </c>
-      <c r="B61" s="8" t="n">
-        <v>240046</v>
+        <v>255673</v>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>252686</v>
-      </c>
-      <c r="B62" s="4" t="n">
-        <v>310</v>
+        <v>255010</v>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>243536</v>
-      </c>
-      <c r="B63" s="7" t="n">
-        <v>240054</v>
+        <v>255618</v>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>243523</v>
-      </c>
-      <c r="B64" s="7" t="n">
-        <v>240054</v>
+        <v>255617</v>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>243535</v>
-      </c>
-      <c r="B65" s="11" t="n">
-        <v>301</v>
+        <v>255709</v>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>243526</v>
-      </c>
-      <c r="B66" s="11" t="n">
-        <v>301</v>
+        <v>260215</v>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>243527</v>
-      </c>
-      <c r="B67" s="11" t="n">
-        <v>301</v>
+        <v>260018</v>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>245089</v>
-      </c>
-      <c r="B68" s="9" t="inlineStr">
+        <v>260270</v>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1100,9 +1123,9 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>245623</v>
-      </c>
-      <c r="B69" s="9" t="inlineStr">
+        <v>260153</v>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1110,51 +1133,59 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>251790</v>
-      </c>
-      <c r="B70" s="3" t="n">
-        <v>40054</v>
+        <v>255388</v>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>252784</v>
-      </c>
-      <c r="B71" s="7" t="n">
-        <v>40055</v>
+        <v>260154</v>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>252785</v>
-      </c>
-      <c r="B72" s="7" t="n">
-        <v>40055</v>
+        <v>254297</v>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>251231</v>
-      </c>
-      <c r="B73" s="5" t="inlineStr">
-        <is>
-          <t>40034 (esterno)</t>
+        <v>260023</v>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>251685</v>
-      </c>
-      <c r="B74" s="3" t="n">
-        <v>40054</v>
+        <v>255561</v>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>252547</v>
-      </c>
-      <c r="B75" s="9" t="inlineStr">
+        <v>255637</v>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1162,9 +1193,499 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>252517</v>
-      </c>
-      <c r="B76" s="9" t="inlineStr">
+        <v>260272</v>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>260061</v>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>260064</v>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>260070</v>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>255548</v>
+      </c>
+      <c r="B80" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>260071</v>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>255565</v>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>260046</v>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>255440</v>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>260204</v>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>260203</v>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>260063</v>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>260139</v>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>255564</v>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>260006</v>
+      </c>
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>260062</v>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>254199</v>
+      </c>
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>260082</v>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>260035</v>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>255796</v>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>255197</v>
+      </c>
+      <c r="B96" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>255190</v>
+      </c>
+      <c r="B97" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>255182</v>
+      </c>
+      <c r="B98" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>255799</v>
+      </c>
+      <c r="B99" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>255710</v>
+      </c>
+      <c r="B100" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>255583</v>
+      </c>
+      <c r="B101" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="n">
+        <v>255608</v>
+      </c>
+      <c r="B102" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n">
+        <v>255482</v>
+      </c>
+      <c r="B103" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n">
+        <v>253788</v>
+      </c>
+      <c r="B104" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n">
+        <v>260296</v>
+      </c>
+      <c r="B105" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>255412</v>
+      </c>
+      <c r="B106" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>255411</v>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>260144</v>
+      </c>
+      <c r="B108" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>255409</v>
+      </c>
+      <c r="B109" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>255410</v>
+      </c>
+      <c r="B110" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>255008</v>
+      </c>
+      <c r="B111" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n">
+        <v>260029</v>
+      </c>
+      <c r="B112" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n">
+        <v>255169</v>
+      </c>
+      <c r="B113" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
+        <v>260261</v>
+      </c>
+      <c r="B114" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n">
+        <v>260065</v>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
+        <v>255611</v>
+      </c>
+      <c r="B116" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
+        <v>255562</v>
+      </c>
+      <c r="B117" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
+        <v>255554</v>
+      </c>
+      <c r="B118" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n">
+        <v>255546</v>
+      </c>
+      <c r="B119" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n">
+        <v>255549</v>
+      </c>
+      <c r="B120" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n">
+        <v>255563</v>
+      </c>
+      <c r="B121" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n">
+        <v>255558</v>
+      </c>
+      <c r="B122" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n">
+        <v>255557</v>
+      </c>
+      <c r="B123" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n">
+        <v>255553</v>
+      </c>
+      <c r="B124" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n">
+        <v>255555</v>
+      </c>
+      <c r="B125" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>